<commit_message>
Initial SAAM Part I implementation
</commit_message>
<xml_diff>
--- a/Template-Part-I-FILLED.xlsx
+++ b/Template-Part-I-FILLED.xlsx
@@ -688,10 +688,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07592064351458019</v>
+        <v>0.0670820558878524</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.07647769141157409</v>
+        <v>0.0794583733751737</v>
       </c>
       <c r="E3" s="22" t="n">
         <v>41640</v>
@@ -700,7 +700,7 @@
         <v>-0.0435349935811963</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>0.0073117259102161</v>
+        <v>-0.0287515686902544</v>
       </c>
     </row>
     <row r="4">
@@ -713,7 +713,7 @@
         <v>0.1291407141705315</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.1193366421989936</v>
+        <v>0.1154979005218071</v>
       </c>
       <c r="E4" s="9" t="n">
         <v>41671</v>
@@ -722,7 +722,7 @@
         <v>0.019246991751624</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.0263700625318461</v>
+        <v>0.0520933741461129</v>
       </c>
     </row>
     <row r="5">
@@ -735,7 +735,7 @@
         <v>1.179584958580808</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.224807136498969</v>
+        <v>1.503057314399208</v>
       </c>
       <c r="E5" s="9" t="n">
         <v>41699</v>
@@ -744,7 +744,7 @@
         <v>0.0026683714969575</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>-0.0021247135184742</v>
+        <v>0.0171999188269799</v>
       </c>
     </row>
     <row r="6">
@@ -754,10 +754,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.5878908445118739</v>
+        <v>0.4715005344785024</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.6408567394082338</v>
+        <v>0.6149194364167639</v>
       </c>
       <c r="E6" s="9" t="n">
         <v>41730</v>
@@ -766,7 +766,7 @@
         <v>-0.0068666427142612</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>-0.0250346010696118</v>
+        <v>-0.0138280133872863</v>
       </c>
     </row>
     <row r="7">
@@ -779,7 +779,7 @@
         <v>-0.1075897946467893</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.1260560062858658</v>
+        <v>-0.1242717964152482</v>
       </c>
       <c r="E7" s="9" t="n">
         <v>41760</v>
@@ -788,7 +788,7 @@
         <v>0.0303178144934912</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.0185390105750233</v>
+        <v>0.0551363227448278</v>
       </c>
     </row>
     <row r="8">
@@ -801,7 +801,7 @@
         <v>0.130681155663674</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.098436470869745</v>
+        <v>0.09832976236810401</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>41791</v>
@@ -810,7 +810,7 @@
         <v>0.0321672383779624</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.0721005493939445</v>
+        <v>0.0464646570539367</v>
       </c>
     </row>
     <row r="9">
@@ -836,7 +836,7 @@
         <v>0.0218518833323933</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.028193212087409</v>
+        <v>0.0145399272475348</v>
       </c>
     </row>
     <row r="10">
@@ -847,7 +847,7 @@
         <v>-0.0118456577284512</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.0655596340963976</v>
+        <v>0.0186444934104972</v>
       </c>
     </row>
     <row r="11">
@@ -858,7 +858,7 @@
         <v>-0.0364315926541183</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-0.0420657348976355</v>
+        <v>-0.0283711875282875</v>
       </c>
     </row>
     <row r="12">
@@ -870,7 +870,7 @@
         <v>0.008401628532876701</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.014939444038751</v>
+        <v>0.0273074749854677</v>
       </c>
     </row>
     <row r="13">
@@ -881,7 +881,7 @@
         <v>-0.009357413058741</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>-0.0454793723045134</v>
+        <v>-0.007945660700164</v>
       </c>
     </row>
     <row r="14">
@@ -892,7 +892,7 @@
         <v>-0.0139599903273446</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>-0.0145396609914625</v>
+        <v>-0.0177158807715862</v>
       </c>
     </row>
     <row r="15">
@@ -903,7 +903,7 @@
         <v>0.0187933362315639</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.0451007745902745</v>
+        <v>0.0605192801397153</v>
       </c>
     </row>
     <row r="16">
@@ -914,7 +914,7 @@
         <v>0.0482112925890249</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>8.689791743290065e-05</v>
+        <v>0.0033634523149509</v>
       </c>
     </row>
     <row r="17">
@@ -925,7 +925,7 @@
         <v>0.008504657454357301</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.0113628041116133</v>
+        <v>0.0068195056624802</v>
       </c>
     </row>
     <row r="18">
@@ -936,7 +936,7 @@
         <v>0.0434155333491115</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.0352955204381012</v>
+        <v>0.030106299647049</v>
       </c>
     </row>
     <row r="19">
@@ -947,7 +947,7 @@
         <v>-0.0004879380389377</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.0057718622310486</v>
+        <v>0.005014841359876</v>
       </c>
     </row>
     <row r="20">
@@ -955,10 +955,10 @@
         <v>42156</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.0245044231952044</v>
+        <v>-0.0245044231952045</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>-0.0132447845038637</v>
+        <v>-0.0071247087726951</v>
       </c>
     </row>
     <row r="21">
@@ -969,7 +969,7 @@
         <v>-0.005767258961163</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.0545491408977184</v>
+        <v>0.0362841901551112</v>
       </c>
     </row>
     <row r="22">
@@ -980,7 +980,7 @@
         <v>-0.07549531951551471</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>-0.0537660072399215</v>
+        <v>-0.0472147327940783</v>
       </c>
     </row>
     <row r="23">
@@ -991,7 +991,7 @@
         <v>-0.0530632295876283</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>-0.0270984142884067</v>
+        <v>0.0407765990677275</v>
       </c>
     </row>
     <row r="24">
@@ -999,10 +999,10 @@
         <v>42278</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0886699838442486</v>
+        <v>0.0886699838442485</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.0600628115908171</v>
+        <v>0.0750256045116007</v>
       </c>
     </row>
     <row r="25">
@@ -1013,7 +1013,7 @@
         <v>-0.0103350477922475</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>-0.0300828483537769</v>
+        <v>-0.0394903519580411</v>
       </c>
     </row>
     <row r="26">
@@ -1024,7 +1024,7 @@
         <v>0.0099641843676856</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.0324011277300471</v>
+        <v>0.0602235604219342</v>
       </c>
     </row>
     <row r="27">
@@ -1032,10 +1032,10 @@
         <v>42370</v>
       </c>
       <c r="F27" t="n">
-        <v>-0.080685356286335</v>
+        <v>-0.08068535628633509</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>-0.050614753318023</v>
+        <v>-0.0401883522945897</v>
       </c>
     </row>
     <row r="28">
@@ -1046,7 +1046,7 @@
         <v>-0.0135581254727204</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.0117690433457753</v>
+        <v>0.0158996618428314</v>
       </c>
     </row>
     <row r="29">
@@ -1054,10 +1054,10 @@
         <v>42430</v>
       </c>
       <c r="F29" t="n">
-        <v>0.06868755891126641</v>
+        <v>0.0686875589112665</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.0556594799486024</v>
+        <v>0.0495512569409307</v>
       </c>
     </row>
     <row r="30">
@@ -1068,7 +1068,7 @@
         <v>0.0316511218767039</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.0380509773655415</v>
+        <v>0.0188467333710436</v>
       </c>
     </row>
     <row r="31">
@@ -1079,7 +1079,7 @@
         <v>-0.0139600690169181</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>-0.0129270072015747</v>
+        <v>0.0029268720371331</v>
       </c>
     </row>
     <row r="32">
@@ -1090,7 +1090,7 @@
         <v>-0.0107078714833797</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.0516512914968159</v>
+        <v>0.0158541384114471</v>
       </c>
     </row>
     <row r="33">
@@ -1101,7 +1101,7 @@
         <v>0.0612765845658077</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.0453675458544198</v>
+        <v>0.0541537488726163</v>
       </c>
     </row>
     <row r="34">
@@ -1112,7 +1112,7 @@
         <v>0.0008255420572559</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>-0.0331216495189693</v>
+        <v>-0.024079270526214</v>
       </c>
     </row>
     <row r="35">
@@ -1123,7 +1123,7 @@
         <v>0.0181536535648113</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.0145823515732836</v>
+        <v>0.0256669696860347</v>
       </c>
     </row>
     <row r="36">
@@ -1134,7 +1134,7 @@
         <v>0.0021874200449166</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>-0.0159838373687071</v>
+        <v>-0.0013180637944866</v>
       </c>
     </row>
     <row r="37">
@@ -1145,7 +1145,7 @@
         <v>-0.0193904334051159</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>-0.0404610979921663</v>
+        <v>-0.0375903651223152</v>
       </c>
     </row>
     <row r="38">
@@ -1156,7 +1156,7 @@
         <v>0.0041856303132661</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0.016614432743491</v>
+        <v>-0.014255018075839</v>
       </c>
     </row>
     <row r="39">
@@ -1167,7 +1167,7 @@
         <v>0.0440280283249324</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.0562571603277339</v>
+        <v>0.0490613440451728</v>
       </c>
     </row>
     <row r="40">
@@ -1178,7 +1178,7 @@
         <v>0.0202206544130379</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.0234754124758861</v>
+        <v>0.0077573797731842</v>
       </c>
     </row>
     <row r="41">
@@ -1189,7 +1189,7 @@
         <v>0.0074971345141355</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.0174491716920261</v>
+        <v>0.0184946234971113</v>
       </c>
     </row>
     <row r="42">
@@ -1200,7 +1200,7 @@
         <v>0.0069527467047144</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.008424784593919</v>
+        <v>0.0039226656247632</v>
       </c>
     </row>
     <row r="43">
@@ -1211,7 +1211,7 @@
         <v>0.0215623610036581</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.0333621655713807</v>
+        <v>0.0443775644276037</v>
       </c>
     </row>
     <row r="44">
@@ -1222,7 +1222,7 @@
         <v>0.0117897180733099</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>-0.0014367916914826</v>
+        <v>0.0021103486769346</v>
       </c>
     </row>
     <row r="45">
@@ -1233,7 +1233,7 @@
         <v>0.0291124290491594</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.0193822193868354</v>
+        <v>0.0170563316806201</v>
       </c>
     </row>
     <row r="46">
@@ -1244,7 +1244,7 @@
         <v>0.0009695412676496001</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>-0.009651220818628301</v>
+        <v>-0.009151411715928299</v>
       </c>
     </row>
     <row r="47">
@@ -1255,7 +1255,7 @@
         <v>0.009010002824520601</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>-0.0080649425366183</v>
+        <v>-0.0111370478662533</v>
       </c>
     </row>
     <row r="48">
@@ -1266,7 +1266,7 @@
         <v>0.0359279854803487</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.0306868152833328</v>
+        <v>0.0196873112697769</v>
       </c>
     </row>
     <row r="49">
@@ -1277,7 +1277,7 @@
         <v>0.0242737538807348</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.0271000723770546</v>
+        <v>0.0277792357849402</v>
       </c>
     </row>
     <row r="50">
@@ -1288,7 +1288,7 @@
         <v>0.0111202132151878</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.0043679838603794</v>
+        <v>-0.0097551979958664</v>
       </c>
     </row>
     <row r="51">
@@ -1299,7 +1299,7 @@
         <v>0.0475087345593656</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.0198166008230914</v>
+        <v>0.0324951451065878</v>
       </c>
     </row>
     <row r="52">
@@ -1310,7 +1310,7 @@
         <v>-0.022999564396508</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>-0.0164772175451688</v>
+        <v>-0.0136683878850766</v>
       </c>
     </row>
     <row r="53">
@@ -1321,7 +1321,7 @@
         <v>-0.0254556263632574</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>-0.0041681958045044</v>
+        <v>-0.0014156455627489</v>
       </c>
     </row>
     <row r="54">
@@ -1332,7 +1332,7 @@
         <v>0.0127323274109773</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.0191132952846775</v>
+        <v>0.0008442643548647</v>
       </c>
     </row>
     <row r="55">
@@ -1343,7 +1343,7 @@
         <v>-0.0083947435344192</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>-0.0173209804754136</v>
+        <v>-0.0013775519625561</v>
       </c>
     </row>
     <row r="56">
@@ -1354,7 +1354,7 @@
         <v>-0.022661244433913</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>-0.0146651941870042</v>
+        <v>-0.0121122899673803</v>
       </c>
     </row>
     <row r="57">
@@ -1365,7 +1365,7 @@
         <v>0.0107465930998898</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.008685423720944101</v>
+        <v>0.0051946767640506</v>
       </c>
     </row>
     <row r="58">
@@ -1376,7 +1376,7 @@
         <v>-0.006414756637926</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>-0.0025402450567484</v>
+        <v>-0.0014727434172006</v>
       </c>
     </row>
     <row r="59">
@@ -1387,7 +1387,7 @@
         <v>0.0191073189557145</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.0207181409331005</v>
+        <v>0.0179223587264144</v>
       </c>
     </row>
     <row r="60">
@@ -1398,7 +1398,7 @@
         <v>-0.0841284269157723</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>-0.0543966519193692</v>
+        <v>-0.054838513711146</v>
       </c>
     </row>
     <row r="61">
@@ -1409,7 +1409,7 @@
         <v>0.0151763507552339</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.0042580808519171</v>
+        <v>-0.002187665570733</v>
       </c>
     </row>
     <row r="62">
@@ -1420,7 +1420,7 @@
         <v>-0.0506309602993229</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>-0.0243800519351656</v>
+        <v>-0.0143540674099991</v>
       </c>
     </row>
     <row r="63">
@@ -1431,7 +1431,7 @@
         <v>0.0607248601107742</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.0332399098460305</v>
+        <v>0.036135231733537</v>
       </c>
     </row>
     <row r="64">
@@ -1442,7 +1442,7 @@
         <v>0.011955783721321</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.0023076638617248</v>
+        <v>-0.0043330393907573</v>
       </c>
     </row>
     <row r="65">
@@ -1453,7 +1453,7 @@
         <v>0.0109285558175756</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>-0.0166860920866494</v>
+        <v>-0.0192111803025797</v>
       </c>
     </row>
     <row r="66">
@@ -1464,7 +1464,7 @@
         <v>0.0146681314872442</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>-0.0303331890987715</v>
+        <v>-0.0280489285026653</v>
       </c>
     </row>
     <row r="67">
@@ -1475,7 +1475,7 @@
         <v>-0.0390842445388862</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>-0.0255406130038076</v>
+        <v>-0.0273539905738265</v>
       </c>
     </row>
     <row r="68">
@@ -1486,7 +1486,7 @@
         <v>0.0439558404804037</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.0101655612431647</v>
+        <v>0.0123629614220318</v>
       </c>
     </row>
     <row r="69">
@@ -1497,7 +1497,7 @@
         <v>-0.0029648380701892</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.0013036132535337</v>
+        <v>-0.0024646483191007</v>
       </c>
     </row>
     <row r="70">
@@ -1508,7 +1508,7 @@
         <v>-0.026484400721349</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>-0.025743961016486</v>
+        <v>-0.0280017519296128</v>
       </c>
     </row>
     <row r="71">
@@ -1519,7 +1519,7 @@
         <v>0.029704659620727</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.0205459497795412</v>
+        <v>0.0284686051457225</v>
       </c>
     </row>
     <row r="72">
@@ -1527,10 +1527,10 @@
         <v>43739</v>
       </c>
       <c r="F72" t="n">
-        <v>0.0416171083855397</v>
+        <v>0.0416171083855398</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.0221438749308524</v>
+        <v>0.0219925914637798</v>
       </c>
     </row>
     <row r="73">
@@ -1541,7 +1541,7 @@
         <v>0.0016869720522591</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>0.0007045151235149</v>
+        <v>-7.001846893496123e-05</v>
       </c>
     </row>
     <row r="74">
@@ -1552,7 +1552,7 @@
         <v>0.024648829860994</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.0316965724263908</v>
+        <v>0.0268849732463479</v>
       </c>
     </row>
     <row r="75">
@@ -1563,7 +1563,7 @@
         <v>-0.0179598865111262</v>
       </c>
       <c r="G75" s="2" t="n">
-        <v>-0.0279770478828585</v>
+        <v>-0.0237718602131903</v>
       </c>
     </row>
     <row r="76">
@@ -1574,7 +1574,7 @@
         <v>-0.0827545264983742</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>-0.070081472441944</v>
+        <v>-0.0589729661281852</v>
       </c>
     </row>
     <row r="77">
@@ -1585,7 +1585,7 @@
         <v>-0.1075897946467893</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>-0.0734076181032474</v>
+        <v>-0.0784991160058835</v>
       </c>
     </row>
     <row r="78">
@@ -1596,7 +1596,7 @@
         <v>0.0654031263308212</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.062256691416908</v>
+        <v>0.0692705259174899</v>
       </c>
     </row>
     <row r="79">
@@ -1607,7 +1607,7 @@
         <v>0.0360976569587131</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>-0.0068668526855685</v>
+        <v>-0.0101542430125601</v>
       </c>
     </row>
     <row r="80">
@@ -1618,7 +1618,7 @@
         <v>0.0206342925218138</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>-0.011501389453573</v>
+        <v>-0.0061225733180612</v>
       </c>
     </row>
     <row r="81">
@@ -1629,7 +1629,7 @@
         <v>-0.0075143424968535</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>-0.0248176280506953</v>
+        <v>-0.008549283008290399</v>
       </c>
     </row>
     <row r="82">
@@ -1640,7 +1640,7 @@
         <v>0.0646055240202412</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>0.0496406277401132</v>
+        <v>0.0381851599550607</v>
       </c>
     </row>
     <row r="83">
@@ -1651,7 +1651,7 @@
         <v>-0.011691058279204</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>-0.016908773551841</v>
+        <v>-0.0187781335998686</v>
       </c>
     </row>
     <row r="84">
@@ -1662,7 +1662,7 @@
         <v>-0.0123324731874683</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>-0.0277999052765775</v>
+        <v>-0.0270284998594713</v>
       </c>
     </row>
     <row r="85">
@@ -1673,7 +1673,7 @@
         <v>0.130681155663674</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>0.0523301491059622</v>
+        <v>0.0552894543162445</v>
       </c>
     </row>
     <row r="86">
@@ -1684,7 +1684,7 @@
         <v>0.0444317954232345</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>0.017140731487109</v>
+        <v>0.0066955889512044</v>
       </c>
     </row>
     <row r="87">
@@ -1695,7 +1695,7 @@
         <v>-0.0048351013302278</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>0.0302995298357336</v>
+        <v>0.0314618326420796</v>
       </c>
     </row>
     <row r="88">
@@ -1706,7 +1706,7 @@
         <v>0.0232990132743903</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>-0.0094551358450887</v>
+        <v>-0.0170230997504482</v>
       </c>
     </row>
     <row r="89">
@@ -1717,7 +1717,7 @@
         <v>0.0153935873574069</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>0.0595883207831417</v>
+        <v>0.0287623113524269</v>
       </c>
     </row>
     <row r="90">
@@ -1728,7 +1728,7 @@
         <v>-0.0007648688726008</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>-0.0164097602668938</v>
+        <v>-0.0024991770919677</v>
       </c>
     </row>
     <row r="91">
@@ -1739,7 +1739,7 @@
         <v>0.0209556919666648</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>-0.0079340875686627</v>
+        <v>0.0132933222736635</v>
       </c>
     </row>
     <row r="92">
@@ -1750,7 +1750,7 @@
         <v>-0.008607642719922299</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>0.0023644064668248</v>
+        <v>-0.0007642147858891</v>
       </c>
     </row>
     <row r="93">
@@ -1761,7 +1761,7 @@
         <v>-0.0163879310489994</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>0.0110906753833523</v>
+        <v>0.0060275862763568</v>
       </c>
     </row>
     <row r="94">
@@ -1772,7 +1772,7 @@
         <v>0.0235472672692028</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0.029687071489735</v>
+        <v>0.0218596291197615</v>
       </c>
     </row>
     <row r="95">
@@ -1783,7 +1783,7 @@
         <v>0.0108641614297038</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>0.0176817551589558</v>
+        <v>0.0121218903641477</v>
       </c>
     </row>
     <row r="96">
@@ -1794,7 +1794,7 @@
         <v>-0.0111454861585684</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>-0.0028927131860375</v>
+        <v>-0.0076368904460683</v>
       </c>
     </row>
     <row r="97">
@@ -1805,7 +1805,7 @@
         <v>-0.0356982050721316</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>-0.0220641911567495</v>
+        <v>-0.010420070984226</v>
       </c>
     </row>
     <row r="98">
@@ -1816,7 +1816,7 @@
         <v>0.028328195448495</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>0.0004960581290341</v>
+        <v>0.0146540895698679</v>
       </c>
     </row>
     <row r="99">
@@ -1827,7 +1827,7 @@
         <v>-0.036800243514807</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>-0.0143008259195349</v>
+        <v>-0.0142503911262826</v>
       </c>
     </row>
     <row r="100">
@@ -1838,7 +1838,7 @@
         <v>0.0011377458853106</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>0.0217526031550754</v>
+        <v>0.0199670118068595</v>
       </c>
     </row>
     <row r="101">
@@ -1849,7 +1849,7 @@
         <v>0.015783214618301</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>-0.0345245375913351</v>
+        <v>-0.0339305708209424</v>
       </c>
     </row>
     <row r="102">
@@ -1857,10 +1857,10 @@
         <v>44652</v>
       </c>
       <c r="F102" t="n">
-        <v>-0.0677131276168875</v>
+        <v>-0.0677131276168874</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>-0.0327726346854507</v>
+        <v>-0.0273126207578517</v>
       </c>
     </row>
     <row r="103">
@@ -1871,7 +1871,7 @@
         <v>0.00698188673958</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>0.0356539480694404</v>
+        <v>0.0385035338181791</v>
       </c>
     </row>
     <row r="104">
@@ -1882,7 +1882,7 @@
         <v>-0.0714494434963429</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>-0.0635146597221998</v>
+        <v>-0.06324777124982429</v>
       </c>
     </row>
     <row r="105">
@@ -1893,7 +1893,7 @@
         <v>0.0432374307202487</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>0.0317407543582558</v>
+        <v>0.0331656275092946</v>
       </c>
     </row>
     <row r="106">
@@ -1904,7 +1904,7 @@
         <v>-0.0199187084572835</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>-0.0052044176615378</v>
+        <v>-0.0050043110185632</v>
       </c>
     </row>
     <row r="107">
@@ -1915,7 +1915,7 @@
         <v>-0.09872846341438581</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>-0.0575898204924272</v>
+        <v>-0.0573195286108208</v>
       </c>
     </row>
     <row r="108">
@@ -1926,7 +1926,7 @@
         <v>0.0154537207239235</v>
       </c>
       <c r="G108" s="2" t="n">
-        <v>-0.0283492715461265</v>
+        <v>-0.0206592802596433</v>
       </c>
     </row>
     <row r="109">
@@ -1934,10 +1934,10 @@
         <v>44866</v>
       </c>
       <c r="F109" t="n">
-        <v>0.1065378940390858</v>
+        <v>0.1065378940390857</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>0.098436470869745</v>
+        <v>0.09832976236810401</v>
       </c>
     </row>
     <row r="110">
@@ -1948,7 +1948,7 @@
         <v>0.0017703432683412</v>
       </c>
       <c r="G110" s="2" t="n">
-        <v>-0.0048364778559603</v>
+        <v>-0.0207041830828527</v>
       </c>
     </row>
     <row r="111">
@@ -1959,7 +1959,7 @@
         <v>0.0652011522005241</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0.03758917169633</v>
+        <v>0.0366481462130185</v>
       </c>
     </row>
     <row r="112">
@@ -1970,7 +1970,7 @@
         <v>-0.0444018309931057</v>
       </c>
       <c r="G112" s="2" t="n">
-        <v>-0.0466684488721246</v>
+        <v>-0.0465416688530787</v>
       </c>
     </row>
     <row r="113">
@@ -1981,7 +1981,7 @@
         <v>0.0286049442421165</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>0.0479309217775114</v>
+        <v>0.0524165648594865</v>
       </c>
     </row>
     <row r="114">
@@ -1992,7 +1992,7 @@
         <v>0.0066046066365428</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>0.0360312432267278</v>
+        <v>0.036151243358694</v>
       </c>
     </row>
     <row r="115">
@@ -2003,7 +2003,7 @@
         <v>-0.0083835386947808</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>-0.0045226259909602</v>
+        <v>-0.0046519504794748</v>
       </c>
     </row>
     <row r="116">
@@ -2014,7 +2014,7 @@
         <v>0.0430608879801947</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>0.0189986364575508</v>
+        <v>0.0194552289981887</v>
       </c>
     </row>
     <row r="117">
@@ -2025,7 +2025,7 @@
         <v>0.0351737329093065</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>0.0355790261506014</v>
+        <v>0.0338357850074215</v>
       </c>
     </row>
     <row r="118">
@@ -2036,7 +2036,7 @@
         <v>-0.0317019609414933</v>
       </c>
       <c r="G118" s="2" t="n">
-        <v>0.0277501028454427</v>
+        <v>0.0272175115272867</v>
       </c>
     </row>
     <row r="119">
@@ -2047,7 +2047,7 @@
         <v>-0.0188549082307113</v>
       </c>
       <c r="G119" s="2" t="n">
-        <v>-0.0137490601075752</v>
+        <v>-0.0144338548124589</v>
       </c>
     </row>
     <row r="120">
@@ -2058,7 +2058,7 @@
         <v>-0.0459503631595632</v>
       </c>
       <c r="G120" s="2" t="n">
-        <v>-0.0271364479007192</v>
+        <v>-0.0289538287806094</v>
       </c>
     </row>
     <row r="121">
@@ -2066,10 +2066,10 @@
         <v>45231</v>
       </c>
       <c r="F121" t="n">
-        <v>0.067990818785886</v>
+        <v>0.0679908187858861</v>
       </c>
       <c r="G121" s="2" t="n">
-        <v>0.0345913573052958</v>
+        <v>0.0336368941465958</v>
       </c>
     </row>
     <row r="122">
@@ -2080,7 +2080,7 @@
         <v>0.0491429755217619</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>-0.1260560062858658</v>
+        <v>-0.1242717964152482</v>
       </c>
     </row>
     <row r="123">
@@ -2091,7 +2091,7 @@
         <v>0.0218027618818123</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>0.0133425418166719</v>
+        <v>0.0130471225033452</v>
       </c>
     </row>
     <row r="124">
@@ -2102,7 +2102,7 @@
         <v>0.0264554865603872</v>
       </c>
       <c r="G124" s="2" t="n">
-        <v>0.0023926055416384</v>
+        <v>0.0020729144706552</v>
       </c>
     </row>
     <row r="125">
@@ -2113,7 +2113,7 @@
         <v>0.0241365225357864</v>
       </c>
       <c r="G125" s="2" t="n">
-        <v>0.0447570902355887</v>
+        <v>0.0448870396945253</v>
       </c>
     </row>
     <row r="126">
@@ -2124,7 +2124,7 @@
         <v>-0.034066183159725</v>
       </c>
       <c r="G126" s="2" t="n">
-        <v>-0.0178481796213439</v>
+        <v>-0.0180438309815904</v>
       </c>
     </row>
     <row r="127">
@@ -2135,7 +2135,7 @@
         <v>0.0116213163305105</v>
       </c>
       <c r="G127" s="2" t="n">
-        <v>0.008360500892512701</v>
+        <v>0.0075019773350089</v>
       </c>
     </row>
     <row r="128">
@@ -2146,7 +2146,7 @@
         <v>-0.0054189705070492</v>
       </c>
       <c r="G128" s="2" t="n">
-        <v>-0.0391191773533319</v>
+        <v>-0.0390905218988838</v>
       </c>
     </row>
     <row r="129">
@@ -2157,7 +2157,7 @@
         <v>0.0465302769809573</v>
       </c>
       <c r="G129" s="2" t="n">
-        <v>0.0775801586553469</v>
+        <v>0.0778920321283479</v>
       </c>
     </row>
     <row r="130">
@@ -2168,7 +2168,7 @@
         <v>0.0146937501815359</v>
       </c>
       <c r="G130" s="2" t="n">
-        <v>-0.001393050587053</v>
+        <v>-0.0017331985613987</v>
       </c>
     </row>
     <row r="131">
@@ -2179,7 +2179,7 @@
         <v>0.0199865103985881</v>
       </c>
       <c r="G131" s="2" t="n">
-        <v>0.0106990011692388</v>
+        <v>0.0107595278656082</v>
       </c>
     </row>
     <row r="132">
@@ -2190,7 +2190,7 @@
         <v>-0.0433874636762671</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>-0.0354747312998371</v>
+        <v>-0.0360610119585291</v>
       </c>
     </row>
     <row r="133">
@@ -2201,7 +2201,7 @@
         <v>0.0047776943894237</v>
       </c>
       <c r="G133" s="2" t="n">
-        <v>0.0452595902487299</v>
+        <v>0.0450887400567218</v>
       </c>
     </row>
     <row r="134">
@@ -2212,7 +2212,7 @@
         <v>-0.010902292498802</v>
       </c>
       <c r="G134" s="2" t="n">
-        <v>-0.0200675083007166</v>
+        <v>-0.0200379823311739</v>
       </c>
     </row>
     <row r="135">
@@ -2223,7 +2223,7 @@
         <v>0.016228420056879</v>
       </c>
       <c r="G135" s="2" t="n">
-        <v>0.0394483078165925</v>
+        <v>0.04297859373411</v>
       </c>
     </row>
     <row r="136">
@@ -2234,7 +2234,7 @@
         <v>-0.0092809624762774</v>
       </c>
       <c r="G136" s="2" t="n">
-        <v>0.0482959173846118</v>
+        <v>0.0489264912281381</v>
       </c>
     </row>
     <row r="137">
@@ -2245,7 +2245,7 @@
         <v>0.0042191259708773</v>
       </c>
       <c r="G137" s="2" t="n">
-        <v>0.0342350956358523</v>
+        <v>0.0373980583438695</v>
       </c>
     </row>
     <row r="138">
@@ -2256,7 +2256,7 @@
         <v>0.0537093125195659</v>
       </c>
       <c r="G138" s="2" t="n">
-        <v>0.0709157634583733</v>
+        <v>0.0749363207391939</v>
       </c>
     </row>
     <row r="139">
@@ -2267,7 +2267,7 @@
         <v>0.0382922269183745</v>
       </c>
       <c r="G139" s="2" t="n">
-        <v>0.0166310443368795</v>
+        <v>0.0184678385216009</v>
       </c>
     </row>
     <row r="140">
@@ -2278,7 +2278,7 @@
         <v>0.021670640724601</v>
       </c>
       <c r="G140" s="2" t="n">
-        <v>0.0452710072673837</v>
+        <v>0.0477679742690069</v>
       </c>
     </row>
     <row r="141">
@@ -2289,7 +2289,7 @@
         <v>-0.0015308589915159</v>
       </c>
       <c r="G141" s="2" t="n">
-        <v>0.0114151184279772</v>
+        <v>0.012694939976014</v>
       </c>
     </row>
     <row r="142">
@@ -2300,7 +2300,7 @@
         <v>0.0614456168602271</v>
       </c>
       <c r="G142" s="2" t="n">
-        <v>0.0374588411575551</v>
+        <v>0.0354718118732805</v>
       </c>
     </row>
     <row r="143">
@@ -2311,7 +2311,7 @@
         <v>0.0149629020739231</v>
       </c>
       <c r="G143" s="2" t="n">
-        <v>0.0211509348853953</v>
+        <v>0.021533670028697</v>
       </c>
     </row>
     <row r="144">
@@ -2322,7 +2322,7 @@
         <v>0.0265252726536321</v>
       </c>
       <c r="G144" s="2" t="n">
-        <v>-0.0001232195856135</v>
+        <v>-0.0016377407785709</v>
       </c>
     </row>
     <row r="145">
@@ -2333,7 +2333,7 @@
         <v>-0.0067052829911501</v>
       </c>
       <c r="G145" s="2" t="n">
-        <v>0.025671184426788</v>
+        <v>0.0259214143527395</v>
       </c>
     </row>
     <row r="146">
@@ -2344,7 +2344,7 @@
         <v>0.0076617247707648</v>
       </c>
       <c r="G146" s="5" t="n">
-        <v>-0.0016893724279862</v>
+        <v>-0.0022332187009084</v>
       </c>
     </row>
   </sheetData>

</xml_diff>